<commit_message>
chore: update news radar report 2026-08-03
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-08-03.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-08-03.xlsx
@@ -446,12 +446,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rising Financial Impact of Out-of-Network Claims on Self-Funded Employers</t>
+          <t>Rising Financial Impact Of Out-Of-Network Claims On Self-Funded Employers</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Rising out-of-network healthcare and pharmacy claims are quietly inflating overall employer-sponsored health plan expenditures due to a lack of price transparency and unmanaged billing practices. This matters because unexpected out-of-network costs directly undermine corporate healthcare cost-containment strategies and strain employee benefits budgets. For business operations, self-funded employers must proactively audit network leakage, implement stricter point-of-service navigation tools, and partner with pharmacy benefits managers to curb escalating out-of-pocket and plan liabilities.</t>
+          <t>Rising out-of-network healthcare and pharmacy claims are driving up unexpected expenditures for self-funded employers. This trend significantly strains employer-sponsored benefit budgets by bypassing negotiated network rates and fueling medical and pharmaceutical inflation. For businesses, this requires tighter plan guardrails, enhanced utilization management, and proactive steerage strategies to mitigate escalating financial exposure.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>